<commit_message>
BSI.IT.27.C7: review E07 C7.Sample response file; add E07 review tab and final conclusion
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkbhuDK8NtXvotyEof7sUo
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7_Final_Conclusions_10_Accounts_3.xlsx
+++ b/BSI.IT.27.C7_Final_Conclusions_10_Accounts_3.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conclusions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E07 Sample review" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conclusions'!$A$4:$N$14</definedName>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +48,10 @@
       <b val="1"/>
     </font>
     <font/>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -107,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -131,6 +136,19 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -498,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1431,6 +1449,13 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>E07 response file (BSI.IT.27.C7_E07_C7.Sample.xlsx) reviewed - screenshots agree to the certification and AD data; no result changes. See tab "E07 Sample review". Final: 3 PASS / 7 FAIL.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:N14"/>
   <mergeCells count="1">
@@ -1439,4 +1464,611 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>BSI.IT.27.C7 - Review of process owner response file BSI.IT.27.C7_E07_C7.Sample.xlsx (screenshots + data tabs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Contents: SAMPLE tab (20 screenshots of the 2026 Q2 SOX Manager and CyberArk Manager certification rows per account), Screenshot tab (PowerShell Get-ADUser run 10/13/2026 11:04 AM -&gt; Oct10_2026Users.csv), 4 certification extracts (2026 Q2 SOX Manager 7/27/2026, SOX Owner, CyberArk Manager 8/17/2026, CyberArk Owner 8/27/2026) and the AD user extract. All 2026 Q2 decisions are after the testing period (07/01/2025-06/30/2026) - used as supporting evidence only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Screenshot vs. data tab</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>2026 Q2 decisions (SOX Mgr 7/27 | CyberArk Mgr 8/17 | CyberArk Owner 8/27)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>SailPoint identity / term date</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>AD 10/13/2026 (enabled | employeeNumber)</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>What the E07 file shows</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>Effect on conclusion</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>MIA25142</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Miguel Nieves Nieves</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Agrees (CyberArk 431-433; SOX 98-100)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Approved | Approved | Approved</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>100546241 / 12/31/2024</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>TRUE | 100546241</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Access revoked 8/28/2025 is still held and was approved three more times in 2026 Q2. No removal date, re-grant request or Netwrix event in the file.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Confirms removal not sustained (A6) and re-grant without request (A5-E3). No change.</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>MIA25172</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Juan Hernandez Ruiz</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Agrees (CyberArk 467-468; SOX 140-142)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Approved | Approved | Approved</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>MIA25172 (uncorrelated) / -</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>TRUE | 100546248</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>AD carries HR number 100546248, but SailPoint still certifies the account against itself (identity = MIA25172), so the reviewer saw no HR identity. Revoked access still held.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Confirms A6 / A5-E3 and the HR-correlation gap (AD has the ID, SailPoint does not). No change.</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>MIA25175</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Hernandez Acevedo</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Agrees (CyberArk 469-471; SOX 143-145)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Approved | Approved | Approved</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>MIA25175 (uncorrelated) / -</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>TRUE | 100546251</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Same as MIA25172 - AD has HR number 100546251; SailPoint identity uncorrelated. Revoked access still held.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Confirms A6 / A5-E3. No change.</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>X453396</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Juan Fernando Perez Peralta</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Agrees (CyberArk 443-445; SOX 110-112)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Approved | Approved | Approved</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>100611758 / -</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>TRUE | 100611758</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Revoked access still held and re-approved. No re-grant request.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Confirms A6 / A5-E3. No change.</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>MIA25103</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Ivan Ramirez Gonzalez</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Agrees (CyberArk 419-421; SOX 86-88)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Approved | Approved | Approved</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>100531048 / 12/31/2024</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>FALSE | 100531048</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Admin account MIA25103 still DISABLED, yet CISCO/ISE admin access approved 3 more times. Same person has an ENABLED personal account x223865 (100531048) - works daily without the admin account.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Strengthens A5-E1: privileged access is not used or needed (4.2.5.1, 4.2.3.1); the exception repeats in 2026 Q2. No change.</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>MIA25104</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Jefferson Paez Venegas</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Agrees (CyberArk 422-424; SOX 89-91)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Approved | Approved | Approved</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>100531049 / 12/31/2024</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>TRUE | 100531049</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Enabled, correlated to HR, consistent approvals. Stale term date 12/31/2024 still shown to reviewers in 2026 Q2.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Supports PASS (E2 cleared by Fieldglass).</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>MIA25105</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>David Serrano Aguirre</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Agrees (CyberArk 425-427; SOX 92-94)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Approved | Approved | Approved</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>100531050 / 12/31/2024</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>TRUE | 100531050</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Enabled, correlated, consistent approvals. Stale term date still shown.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Supports PASS.</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>MIA25106</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Maiko Vazquez Arias</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Agrees (CyberArk 428-430; SOX 95-97)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Approved | Approved | Approved</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>100531051 / 12/31/2024</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>TRUE | 100531051</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Enabled, correlated, consistent approvals. Stale term date still shown.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Supports PASS.</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>MIA25249</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Richard Harris</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Agrees (CyberArk 437-439; SOX 104-106)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Approved | Approved | Approved</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>100592069 / 12/31/2024</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>TRUE | 100592069</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Account ENABLED on 10/13/2026 - confirms it was re-enabled after the 4/2/2026 disablement. The file has no request/ticket for the re-enable and no reason for the disablement; the Get-ADUser query does not pull whenChanged, lastLogonDate or memberOf.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>2025 Q3 passes. 2026 Q1 A5-E1 and unevidenced re-enable (4.2.3.4) stand. No change.</t>
+        </is>
+      </c>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>MIA25250</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Kevin Ackley</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Agrees (CyberArk 434-436; SOX 101-103)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Approved | Approved | Approved</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>100592068 / 12/31/2024</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>TRUE | blank (employeeID also blank)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Re-enabled after 4/3/2026 (enabled 10/13/2026), no request. AD admin account has no employeeID/Number; HR number 100592068 sits on personal account x375759. SAMPLE tab Identity for this row is typed in (100592068) instead of the VLOOKUP formula used for the other 9 - the lookup would return nothing.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Confirms re-enable without request and AD not synchronized with HR (4.2.1.1). No change.</t>
+        </is>
+      </c>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Overall conclusion: the E07 file does not change any result. FINAL: 3 PASS (MIA25104, MIA25105, MIA25106) / 7 FAIL (MIA25142, MIA25172, MIA25175, X453396, MIA25103, MIA25249, MIA25250).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Screenshots: all 20 SAMPLE-tab screenshots match the rows in the 2026Q2PamBsiSox-Manager and 2026Q2BsiPamCyberark-Manager tabs (same row numbers, decision, identity and entitlement). They show 2026 Q2 decisions only - nothing for the in-period samples (8/28/2025, 4/30/2026), no removal dates, no request tickets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Reliability of the certification extracts: "Account Status" = "Account Removed" on every row of all four tabs (680 + 3,685 + 188 + 336 rows), including accounts that are enabled in AD, so this field is not reliable and was not used. "Termination Date" still shows 12/31/2024 for the contractors in 2026 Q2 - reviewers were still certifying against the stale SanIAM date (supports the SanIAM-Fieldglass reconciliation observation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Reliability of the AD extract: the PowerShell command and full scope (-Filter *) are visible, so the extract is complete for the attributes selected. The run is dated 10/13/2026 11:04 AM while the file is named Oct10_2026Users - record the extract date as 10/13/2026. The query does not include lastLogonDate, whenChanged or memberOf, so it cannot evidence group membership, disable/re-enable dates or usage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Owner-level certifications (CyberArk Owner, Heredia 8/27/2026; SOX Owner) approved every row (3,685 and 336 rows, 0 revocations) - the second-level review did not catch the disabled or re-granted accounts either.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Still needed to change any FAIL: ServiceNow requests/approvals for the re-grants (MIA25142, MIA25172, MIA25175, X453396) and re-enables (MIA25249, MIA25250); reason for the 4/2-4/3/2026 disablement; Netwrix add/enable events with dates.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A16:I16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
BSI.IT.27.C7: assess process owner 'no revocations / extended' reply; add reply draft
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkbhuDK8NtXvotyEof7sUo
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7_Final_Conclusions_10_Accounts_3.xlsx
+++ b/BSI.IT.27.C7_Final_Conclusions_10_Accounts_3.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -662,12 +662,14 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Response (C7.Sample.xlsx) showed the account in the 2026 Q2 SOX Manager (rows 98-100) and CyberArk Manager (431-433) certifications, all Approved by Borges, Dayam, and AD enabled on 10/10/2026. No removal date, Netwrix log, ServiceNow ticket or explanation for the re-grant was provided. Process owner position: SanIAM shows no change / mover / leaver events.</t>
+          <t>Response (C7.Sample.xlsx) showed the account in the 2026 Q2 SOX Manager (rows 98-100) and CyberArk Manager (431-433) certifications, all Approved by Borges, Dayam, and AD enabled on 10/10/2026. No removal date, Netwrix log, ServiceNow ticket or explanation for the re-grant was provided. Process owner position: SanIAM shows no change / mover / leaver events.
+(5) Process owner reply: 'There are no revocations; access was approved by the manager, so there is no SLA; consultants were extended, which is why they were certified in 2025 and 2026.'</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Not accepted. The response confirms the access is still held and was re-approved; it does not evidence an approved request for the re-grant after the 9/2/2025 removal. Exception stands.</t>
+          <t>Not accepted. The response confirms the access is still held and was re-approved; it does not evidence an approved request for the re-grant after the 9/2/2025 removal. Exception stands.
+(5) NOT ACCEPTED - contradicts the 2025 Q3 certification: the manager REVOKED this account on 8/28/2025 and it was removed from AD (SLA met). The exception is the re-grant without a request (4.2.3.4); a later manager approval does not replace that request. Extension is not relevant (Fieldglass not in scope for this account).</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -739,12 +741,14 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Response showed 2026 Q2 SOX Manager (140-142) and CyberArk Manager (467-468) rows Approved and AD enabled 10/10/2026. No re-grant request, Netwrix event or explanation provided; no explanation for the uncorrelated identity or the ISEAdmin add.</t>
+          <t>Response showed 2026 Q2 SOX Manager (140-142) and CyberArk Manager (467-468) rows Approved and AD enabled 10/10/2026. No re-grant request, Netwrix event or explanation provided; no explanation for the uncorrelated identity or the ISEAdmin add.
+(5) Process owner reply: 'There are no revocations; access was approved by the manager, so there is no SLA; consultants were extended, which is why they were certified in 2025 and 2026.'</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Not accepted. Re-approval in 2026 Q2 confirms the removal was not sustained. Exception stands.</t>
+          <t>Not accepted. Re-approval in 2026 Q2 confirms the removal was not sustained. Exception stands.
+(5) NOT ACCEPTED - contradicts the 2025 Q3 certification: the manager REVOKED this account on 8/28/2025 and it was removed from AD (SLA met). The exception is the re-grant without a request (4.2.3.4); a later manager approval does not replace that request. Extension is not relevant (Fieldglass not in scope for this account).</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -817,12 +821,14 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Response showed 2026 Q2 SOX Manager (143-145) and CyberArk Manager (469-471) rows Approved and AD enabled 10/10/2026. No re-grant request, Netwrix event or explanation provided; no explanation for the uncorrelated identity or the ISEAdmin add.</t>
+          <t>Response showed 2026 Q2 SOX Manager (143-145) and CyberArk Manager (469-471) rows Approved and AD enabled 10/10/2026. No re-grant request, Netwrix event or explanation provided; no explanation for the uncorrelated identity or the ISEAdmin add.
+(5) Process owner reply: 'There are no revocations; access was approved by the manager, so there is no SLA; consultants were extended, which is why they were certified in 2025 and 2026.'</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Not accepted. Exception stands.</t>
+          <t>Not accepted. Exception stands.
+(5) NOT ACCEPTED - contradicts the 2025 Q3 certification: the manager REVOKED this account on 8/28/2025 and it was removed from AD (SLA met). The exception is the re-grant without a request (4.2.3.4); a later manager approval does not replace that request. Extension is not relevant (Fieldglass not in scope for this account).</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -895,12 +901,14 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Response showed 2026 Q2 SOX Manager (110-112) and CyberArk Manager (443-445) rows Approved and AD enabled 10/10/2026. No re-grant request or Netwrix event provided.</t>
+          <t>Response showed 2026 Q2 SOX Manager (110-112) and CyberArk Manager (443-445) rows Approved and AD enabled 10/10/2026. No re-grant request or Netwrix event provided.
+(5) Process owner reply: 'There are no revocations; access was approved by the manager, so there is no SLA; consultants were extended, which is why they were certified in 2025 and 2026.'</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Not accepted. Exception stands.</t>
+          <t>Not accepted. Exception stands.
+(5) NOT ACCEPTED - contradicts the 2025 Q3 certification: the manager REVOKED this account on 8/28/2025 and it was removed from AD (SLA met). The exception is the re-grant without a request (4.2.3.4); a later manager approval does not replace that request. Extension is not relevant (Fieldglass not in scope for this account).</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -971,13 +979,15 @@
       <c r="I9" s="4" t="inlineStr">
         <is>
           <t>(1) 'If the access is approved, what SLA is being measured? The SLA only starts if the access is revoked.' (2) The consultants were extended - that is why they were certified in 2025 and 2026. (3) SanIAM shows no change, mover or leaver events. Fieldglass provided 10/29/2026 (worker SANWK00016501 Open 2024-01-01 to 2027-02-28). No explanation for why the disabled account keeps admin access.
-(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.</t>
+(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.
+(5) Process owner reply: 'There are no revocations; access was approved by the manager, so there is no SLA; consultants were extended, which is why they were certified in 2025 and 2026.'</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
           <t>(1) AGREED - A6 N/A, no SLA exception. (2) SUPPORTED by Fieldglass - E2 cleared. (3) Does not explain approving an account disabled in AD and unused since 10/15/2023. A5-E1 exception stands.
-(4) NOT ACCEPTED - Fieldglass proves the person is an active contractor (who the person is), not that this privileged access is valid or needed (what the account can do). The AD account has been disabled with no logon since 10/15/2023 while the contractor has been working continuously since 2024-01-01 - i.e., the contractor works without this admin account, which shows the CISCO/ISE admin access is not needed (4.2.5.1 least privilege). Active status supports revocation, not approval. FAIL stands.</t>
+(4) NOT ACCEPTED - Fieldglass proves the person is an active contractor (who the person is), not that this privileged access is valid or needed (what the account can do). The AD account has been disabled with no logon since 10/15/2023 while the contractor has been working continuously since 2024-01-01 - i.e., the contractor works without this admin account, which shows the CISCO/ISE admin access is not needed (4.2.5.1 least privilege). Active status supports revocation, not approval. FAIL stands.
+(5) Partly agreed - no revocation and no SLA exception (agreed); extension supported (agreed). Not accepted as clearing the exception: the finding is the approval itself - manager approval is the control being tested, and 4.2.5.1 requires it to confirm the privileged access is valid and needed. Approval of an AD-disabled account unused since 10/15/2023 does not meet that.</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -1048,13 +1058,15 @@
       <c r="I10" s="4" t="inlineStr">
         <is>
           <t>(1) SLA only applies to revoked access. (2) Consultant contract was extended - that is why the account was certified. (3) No change / mover / leaver events in SanIAM. Fieldglass provided 10/29/2026 (worker SANWK00016508 Open 2024-01-01 to 2027-02-28; buyer ref 100531049 = SanIAM identity).
-(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.</t>
+(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.
+(5) Process owner reply: 'There are no revocations; access was approved by the manager, so there is no SLA; consultants were extended, which is why they were certified in 2025 and 2026.'</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
           <t>(1) AGREED - A6 N/A. (2) SUPPORTED by Fieldglass - active on 8/28/2025 and 4/30/2026; IAMS 12/31/2024 is stale. Explanation accepted - no exception.
-(4) AGREED - active Fieldglass engagement is the basis for the PASS (E2 was the only issue).</t>
+(4) AGREED - active Fieldglass engagement is the basis for the PASS (E2 was the only issue).
+(5) AGREED - no revocation, no SLA; extension supported by Fieldglass. Basis for PASS.</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -1124,13 +1136,15 @@
       <c r="I11" s="4" t="inlineStr">
         <is>
           <t>(1) SLA only applies to revoked access. (2) Contract extended. (3) No change / mover / leaver events. Fieldglass provided (worker SANWK00016502 Open 2024-01-01 to 2027-02-28; buyer ref 100531050 = SanIAM identity).
-(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.</t>
+(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.
+(5) Process owner reply: 'There are no revocations; access was approved by the manager, so there is no SLA; consultants were extended, which is why they were certified in 2025 and 2026.'</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
           <t>(1) AGREED. (2) SUPPORTED by Fieldglass. Explanation accepted - no exception.
-(4) AGREED - active Fieldglass engagement is the basis for the PASS (E2 was the only issue).</t>
+(4) AGREED - active Fieldglass engagement is the basis for the PASS (E2 was the only issue).
+(5) AGREED - no revocation, no SLA; extension supported by Fieldglass. Basis for PASS.</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -1200,13 +1214,15 @@
       <c r="I12" s="4" t="inlineStr">
         <is>
           <t>(1) SLA only applies to revoked access. (2) Contract extended. (3) No change / mover / leaver events. Fieldglass provided (worker SANWK00016503 Open 2024-01-01 to 2027-02-28; buyer ref 100531051 = SanIAM identity).
-(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.</t>
+(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.
+(5) Process owner reply: 'There are no revocations; access was approved by the manager, so there is no SLA; consultants were extended, which is why they were certified in 2025 and 2026.'</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
           <t>(1) AGREED. (2) SUPPORTED by Fieldglass. Explanation accepted - no exception.
-(4) AGREED - active Fieldglass engagement is the basis for the PASS (E2 was the only issue).</t>
+(4) AGREED - active Fieldglass engagement is the basis for the PASS (E2 was the only issue).
+(5) AGREED - no revocation, no SLA; extension supported by Fieldglass. Basis for PASS.</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -1276,13 +1292,15 @@
       <c r="I13" s="4" t="inlineStr">
         <is>
           <t>(1) SLA only applies to revoked access. (2) Contract extended. (3) No change / mover / leaver events. Fieldglass provided (worker SANWK00016311 Open 2023-12-28 to 2027-02-28; buyer ref 100592069 = SanIAM identity). No explanation for the 4/2/2026 AD disablement or the re-enable by 10/10/2026.
-(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.</t>
+(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.
+(5) Process owner reply: 'There are no revocations; access was approved by the manager, so there is no SLA; consultants were extended, which is why they were certified in 2025 and 2026.'</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
           <t>(1) AGREED - A6 N/A. (2) SUPPORTED - E2 cleared; 2025 Q3 passes. (3) Does not explain approval on 4/30/2026 of an account disabled since 4/2/2026, or the unevidenced re-enable. A5-E1 exception stands for 2026 Q1.
-(4) PARTIALLY ACCEPTED - active status clears E2 and the 2025 Q3 sample passes. It does not clear 2026 Q1: the exception is that the reviewer approved privileged access on 4/30/2026 for an account disabled in AD since 4/2/2026 without addressing it, and the account was later re-enabled with no request (4.2.3.4). Being active does not explain why the account was disabled or authorize the re-enable. Also, the Fieldglass screenshot shows the current Open period only - not status as of 4/30/2026 or any April 2026 gap, which was specifically requested. FAIL stands for 2026 Q1.</t>
+(4) PARTIALLY ACCEPTED - active status clears E2 and the 2025 Q3 sample passes. It does not clear 2026 Q1: the exception is that the reviewer approved privileged access on 4/30/2026 for an account disabled in AD since 4/2/2026 without addressing it, and the account was later re-enabled with no request (4.2.3.4). Being active does not explain why the account was disabled or authorize the re-enable. Also, the Fieldglass screenshot shows the current Open period only - not status as of 4/30/2026 or any April 2026 gap, which was specifically requested. FAIL stands for 2026 Q1.
+(5) Partly agreed - no revocation and no SLA exception (agreed); extension supported (agreed). Not accepted as clearing the exception: the finding is the approval itself - manager approval is the control being tested, and 4.2.5.1 requires it to confirm the privileged access is valid and needed. Approval of an AD-disabled account (and the later re-enable without request) does not meet that.</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -1352,13 +1370,15 @@
       <c r="I14" s="4" t="inlineStr">
         <is>
           <t>(1) SLA only applies to revoked access. (2) Contract extended. (3) No change / mover / leaver events. Fieldglass provided (worker SANWK00016313 Open 2023-12-28 to 2027-02-28; buyer ref 100592068 = SanIAM identity). No explanation for the 4/3/2026 disablement, the re-enable, or the blank AD employeeNumber.
-(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.</t>
+(4) Follow-up after Fieldglass (10/29/2026): process owner states the account should PASS because the contractor is active in Fieldglass.
+(5) Process owner reply: 'There are no revocations; access was approved by the manager, so there is no SLA; consultants were extended, which is why they were certified in 2025 and 2026.'</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
           <t>(1) AGREED - A6 N/A. (2) SUPPORTED - E2 cleared; 2025 Q3 passes. (3) Does not explain the 2026 Q1 approval of a disabled account or the re-enable. A5-E1 exception stands for 2026 Q1.
-(4) PARTIALLY ACCEPTED - same as MIA25249: active status clears E2 and 2025 Q3 passes; it does not explain the 4/3/2026 disablement, the 4/30/2026 approval of a disabled account, the unevidenced re-enable, or the blank AD employeeNumber. FAIL stands for 2026 Q1.</t>
+(4) PARTIALLY ACCEPTED - same as MIA25249: active status clears E2 and 2025 Q3 passes; it does not explain the 4/3/2026 disablement, the 4/30/2026 approval of a disabled account, the unevidenced re-enable, or the blank AD employeeNumber. FAIL stands for 2026 Q1.
+(5) Partly agreed - no revocation and no SLA exception (agreed); extension supported (agreed). Not accepted as clearing the exception: the finding is the approval itself - manager approval is the control being tested, and 4.2.5.1 requires it to confirm the privileged access is valid and needed. Approval of an AD-disabled account (and the later re-enable without request) does not meet that.</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -1453,6 +1473,13 @@
       <c r="A25" t="inlineStr">
         <is>
           <t>E07 response file (BSI.IT.27.C7_E07_C7.Sample.xlsx) reviewed - screenshots agree to the certification and AD data; no result changes. See tab "E07 Sample review". Final: 3 PASS / 7 FAIL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Process owner reply (no revocations / manager approved / no SLA / consultants extended): SLA and extension points AGREED and already reflected (MIA25104-106 PASS). 'No revocations' is not correct for MIA25142, MIA25172, MIA25175, X453396 - revoked 8/28/2025 in the 2025 Q3 cert and re-granted without request. For MIA25103, MIA25249, MIA25250 the exception is the appropriateness of the approval (4.2.5.1), not revocation/SLA. Result unchanged: 3 PASS / 7 FAIL.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BSI.IT.27.C7: add re-enable requirement for MIA25249/MIA25250 to reply and workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkbhuDK8NtXvotyEof7sUo
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7_Final_Conclusions_10_Accounts_3.xlsx
+++ b/BSI.IT.27.C7_Final_Conclusions_10_Accounts_3.xlsx
@@ -1300,7 +1300,8 @@
         <is>
           <t>(1) AGREED - A6 N/A. (2) SUPPORTED - E2 cleared; 2025 Q3 passes. (3) Does not explain approval on 4/30/2026 of an account disabled since 4/2/2026, or the unevidenced re-enable. A5-E1 exception stands for 2026 Q1.
 (4) PARTIALLY ACCEPTED - active status clears E2 and the 2025 Q3 sample passes. It does not clear 2026 Q1: the exception is that the reviewer approved privileged access on 4/30/2026 for an account disabled in AD since 4/2/2026 without addressing it, and the account was later re-enabled with no request (4.2.3.4). Being active does not explain why the account was disabled or authorize the re-enable. Also, the Fieldglass screenshot shows the current Open period only - not status as of 4/30/2026 or any April 2026 gap, which was specifically requested. FAIL stands for 2026 Q1.
-(5) Partly agreed - no revocation and no SLA exception (agreed); extension supported (agreed). Not accepted as clearing the exception: the finding is the approval itself - manager approval is the control being tested, and 4.2.5.1 requires it to confirm the privileged access is valid and needed. Approval of an AD-disabled account (and the later re-enable without request) does not meet that.</t>
+(5) Partly agreed - no revocation and no SLA exception (agreed); extension supported (agreed). Not accepted as clearing the exception: the finding is the approval itself - manager approval is the control being tested, and 4.2.5.1 requires it to confirm the privileged access is valid and needed. Approval of an AD-disabled account (and the later re-enable without request) does not meet that.
+(6) Re-enable: re-enabling a disabled account restores privileged access, so it is provisioning and needs an approved request (4.2.3.4). The quoted policy gives no exemption based on how long the account was disabled. The disablement was not short: last logon 11/17/2025, disabled 4/2/2026 (~4.5 months unused, consistent with a 90-day inactivity disablement under 4.2.3.1), still disabled at the 4/30/2026 approval, and first seen enabled again 10/13/2026 (exact re-enable date unknown - the AD extract has no whenChanged). A documented reactivation under a policy procedure could reduce the re-enable point to an observation; the 4.2.5.1 approval exception stands either way.</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -1324,7 +1325,7 @@
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>Reason for the 4/2-4/3/2026 disablement of 9 contractor accounts + approved re-enable request could reduce to an observation. Fieldglass detail ('Go to Details' / work order revision history) showing status as of 4/30/2026 and no April 2026 gap is also needed; active status alone does not change the conclusion.</t>
+          <t>Reason for the 4/2-4/3/2026 disablement of 9 contractor accounts + approved re-enable request could reduce to an observation. Fieldglass detail ('Go to Details' / work order revision history) showing status as of 4/30/2026 and no April 2026 gap is also needed; active status alone does not change the conclusion. Also: date of re-enable (Netwrix/AD event) and the reactivation procedure followed, if the IAM Standard or PAM Procedure defines one.</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1379,8 @@
         <is>
           <t>(1) AGREED - A6 N/A. (2) SUPPORTED - E2 cleared; 2025 Q3 passes. (3) Does not explain the 2026 Q1 approval of a disabled account or the re-enable. A5-E1 exception stands for 2026 Q1.
 (4) PARTIALLY ACCEPTED - same as MIA25249: active status clears E2 and 2025 Q3 passes; it does not explain the 4/3/2026 disablement, the 4/30/2026 approval of a disabled account, the unevidenced re-enable, or the blank AD employeeNumber. FAIL stands for 2026 Q1.
-(5) Partly agreed - no revocation and no SLA exception (agreed); extension supported (agreed). Not accepted as clearing the exception: the finding is the approval itself - manager approval is the control being tested, and 4.2.5.1 requires it to confirm the privileged access is valid and needed. Approval of an AD-disabled account (and the later re-enable without request) does not meet that.</t>
+(5) Partly agreed - no revocation and no SLA exception (agreed); extension supported (agreed). Not accepted as clearing the exception: the finding is the approval itself - manager approval is the control being tested, and 4.2.5.1 requires it to confirm the privileged access is valid and needed. Approval of an AD-disabled account (and the later re-enable without request) does not meet that.
+(6) Re-enable: re-enabling a disabled account restores privileged access, so it is provisioning and needs an approved request (4.2.3.4). The quoted policy gives no exemption based on how long the account was disabled. The disablement was not short: last logon 11/07/2025, disabled 4/3/2026 (~4.5 months unused, consistent with a 90-day inactivity disablement under 4.2.3.1), still disabled at the 4/30/2026 approval, and first seen enabled again 10/13/2026 (exact re-enable date unknown - the AD extract has no whenChanged). A documented reactivation under a policy procedure could reduce the re-enable point to an observation; the 4.2.5.1 approval exception stands either way.</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -1402,7 +1404,7 @@
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>Same as MIA25249; also populate employeeNumber.</t>
+          <t>Same as MIA25249; also populate employeeNumber. Also: date of re-enable (Netwrix/AD event) and the reactivation procedure followed, if the IAM Standard or PAM Procedure defines one.</t>
         </is>
       </c>
     </row>

</xml_diff>